<commit_message>
Auto-generate blog post 2026-09-14
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -1385,12 +1385,12 @@
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>Spoke post — cite established models, add GrowthMax variant</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/ai-maturity-model/</t>
         </is>
       </c>
       <c r="O9" s="5" t="inlineStr">
@@ -9295,7 +9295,12 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-09-14</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>/blog/ai-maturity-model/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-09-16
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -3730,12 +3730,12 @@
       </c>
       <c r="M44" s="5" t="inlineStr">
         <is>
-          <t>Strong existing positioning</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N44" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/how-to-build-an-ai-literacy-program-that-sticks/</t>
         </is>
       </c>
       <c r="O44" s="5" t="inlineStr">
@@ -9338,7 +9338,12 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-09-16</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>/blog/how-to-build-an-ai-literacy-program-that-sticks/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-09-25
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -2323,12 +2323,12 @@
       </c>
       <c r="M23" s="5" t="inlineStr">
         <is>
-          <t>Spoke post (Salesforce, Workday, SAP examples)</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N23" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/ai-agent-integration-connecting-to-existing-systems/</t>
         </is>
       </c>
       <c r="O23" s="5" t="inlineStr">
@@ -9381,7 +9381,12 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-09-25</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>/blog/ai-agent-integration-connecting-to-existing-systems/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-09-28
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -4333,12 +4333,12 @@
       </c>
       <c r="M53" s="5" t="inlineStr">
         <is>
-          <t>Part of new pillar</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N53" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/designing-human-ai-collaboration-that-holds-up/</t>
         </is>
       </c>
       <c r="O53" s="5" t="inlineStr">
@@ -9424,7 +9424,12 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-09-28</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>/blog/designing-human-ai-collaboration-that-holds-up/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-09-30
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -3462,12 +3462,12 @@
       </c>
       <c r="M40" s="5" t="inlineStr">
         <is>
-          <t>Secondary keyword</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N40" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/how-long-ai-implementation-really-takes/</t>
         </is>
       </c>
       <c r="O40" s="5" t="inlineStr">
@@ -9467,7 +9467,12 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-09-30</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>/blog/how-long-ai-implementation-really-takes/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-10-02
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -2658,12 +2658,12 @@
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>Spoke post — eval frameworks, metrics</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N28" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/how-to-evaluate-an-ai-agent-before-you-trust-it/</t>
         </is>
       </c>
       <c r="O28" s="5" t="inlineStr">
@@ -9510,7 +9510,12 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-10-02</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>/blog/how-to-evaluate-an-ai-agent-before-you-trust-it/</t>
         </is>
       </c>
     </row>

</xml_diff>